<commit_message>
Remove node_modules from repo and configure .gitignore
</commit_message>
<xml_diff>
--- a/property_engine.xlsx
+++ b/property_engine.xlsx
@@ -1698,7 +1698,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="278">
   <si>
     <t>id</t>
   </si>
@@ -2238,6 +2238,12 @@
   </si>
   <si>
     <t>TEXT</t>
+  </si>
+  <si>
+    <t>018f3a3a-7002-7000-8000-000000000006</t>
+  </si>
+  <si>
+    <t>has_beinsport</t>
   </si>
   <si>
     <t>attributeId</t>
@@ -3330,7 +3336,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -3549,6 +3555,35 @@
         <v>1</v>
       </c>
       <c r="L6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" t="s">
+        <v>143</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3583,10 +3618,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D1" s="12" t="s">
         <v>111</v>
@@ -3622,7 +3657,7 @@
         <v>131</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D1" s="12" t="s">
         <v>158</v>
@@ -3639,7 +3674,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B2" t="s">
         <v>119</v>
@@ -3662,7 +3697,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B3" t="s">
         <v>119</v>
@@ -3685,7 +3720,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B4" t="s">
         <v>119</v>
@@ -3708,7 +3743,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B5" t="s">
         <v>129</v>
@@ -3731,7 +3766,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B6" t="s">
         <v>129</v>
@@ -3754,7 +3789,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B7" t="s">
         <v>129</v>
@@ -3800,33 +3835,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B2" t="s">
         <v>136</v>
@@ -3840,7 +3875,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B3" t="s">
         <v>136</v>
@@ -3849,12 +3884,12 @@
         <v>177</v>
       </c>
       <c r="D3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B4" t="s">
         <v>139</v>
@@ -3868,7 +3903,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B5" t="s">
         <v>139</v>
@@ -3910,13 +3945,13 @@
         <v>4</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G1" s="14" t="s">
         <v>60</v>
@@ -3924,19 +3959,19 @@
     </row>
     <row r="2" ht="22.05" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F2" s="4" t="b">
         <v>1</v>
@@ -3947,19 +3982,19 @@
     </row>
     <row r="3" ht="22.05" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F3" s="4" t="b">
         <v>0</v>
@@ -4001,27 +4036,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F1" s="14" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>5</v>
@@ -4030,7 +4065,7 @@
         <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>9</v>
@@ -4038,10 +4073,10 @@
     </row>
     <row r="3" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>5</v>
@@ -4050,18 +4085,18 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>31</v>
@@ -4070,7 +4105,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>33</v>
@@ -4078,10 +4113,10 @@
     </row>
     <row r="5" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>31</v>
@@ -4090,18 +4125,18 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>46</v>
@@ -4110,7 +4145,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>48</v>
@@ -4118,10 +4153,10 @@
     </row>
     <row r="7" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>46</v>
@@ -4130,58 +4165,58 @@
         <v>4</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="8" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" ht="22.05" customHeight="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>231</v>
-      </c>
       <c r="E9" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B10" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
@@ -4190,7 +4225,7 @@
         <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F10" t="s">
         <v>24</v>
@@ -4198,10 +4233,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B11" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -4210,18 +4245,18 @@
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C12" t="s">
         <v>25</v>
@@ -4230,18 +4265,18 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C13" t="s">
         <v>25</v>
@@ -4250,7 +4285,7 @@
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F13" t="s">
         <v>29</v>
@@ -4258,10 +4293,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B14" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C14" t="s">
         <v>43</v>
@@ -4270,18 +4305,18 @@
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F14" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B15" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -4290,7 +4325,7 @@
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F15" t="s">
         <v>44</v>
@@ -4298,10 +4333,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B16" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C16" t="s">
         <v>58</v>
@@ -4310,18 +4345,18 @@
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F16" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B17" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C17" t="s">
         <v>58</v>
@@ -4330,7 +4365,7 @@
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F17" t="s">
         <v>59</v>
@@ -4338,90 +4373,90 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B18" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C18" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D18" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E18" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F18" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>253</v>
+      </c>
+      <c r="B19" t="s">
+        <v>250</v>
+      </c>
+      <c r="C19" t="s">
         <v>251</v>
       </c>
-      <c r="B19" t="s">
-        <v>248</v>
-      </c>
-      <c r="C19" t="s">
-        <v>249</v>
-      </c>
       <c r="D19" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E19" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F19" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B20" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C20" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D20" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E20" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F20" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B21" t="s">
+        <v>250</v>
+      </c>
+      <c r="C21" t="s">
         <v>256</v>
       </c>
-      <c r="B21" t="s">
-        <v>248</v>
-      </c>
-      <c r="C21" t="s">
-        <v>254</v>
-      </c>
       <c r="D21" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E21" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F21" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B22" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C22" t="s">
         <v>101</v>
@@ -4430,18 +4465,18 @@
         <v>4</v>
       </c>
       <c r="E22" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F22" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>263</v>
+      </c>
+      <c r="B23" t="s">
         <v>261</v>
-      </c>
-      <c r="B23" t="s">
-        <v>259</v>
       </c>
       <c r="C23" t="s">
         <v>101</v>
@@ -4450,18 +4485,18 @@
         <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F23" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B24" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C24" t="s">
         <v>101</v>
@@ -4470,7 +4505,7 @@
         <v>4</v>
       </c>
       <c r="E24" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F24" t="s">
         <v>103</v>
@@ -4478,10 +4513,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B25" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C25" t="s">
         <v>101</v>
@@ -4490,7 +4525,7 @@
         <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F25" t="s">
         <v>104</v>
@@ -4498,90 +4533,90 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B26" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C26" t="s">
         <v>113</v>
       </c>
       <c r="D26" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E26" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F26" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B27" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C27" t="s">
         <v>113</v>
       </c>
       <c r="D27" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E27" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F27" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B28" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C28" t="s">
         <v>116</v>
       </c>
       <c r="D28" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E28" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F28" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B29" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C29" t="s">
         <v>116</v>
       </c>
       <c r="D29" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E29" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F29" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B30" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C30" t="s">
         <v>136</v>
@@ -4590,18 +4625,18 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F30" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>274</v>
+      </c>
+      <c r="B31" t="s">
         <v>272</v>
-      </c>
-      <c r="B31" t="s">
-        <v>270</v>
       </c>
       <c r="C31" t="s">
         <v>136</v>
@@ -4610,7 +4645,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F31" t="s">
         <v>137</v>
@@ -4618,10 +4653,10 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B32" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C32" t="s">
         <v>139</v>
@@ -4630,18 +4665,18 @@
         <v>4</v>
       </c>
       <c r="E32" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F32" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B33" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C33" t="s">
         <v>139</v>
@@ -4650,7 +4685,7 @@
         <v>4</v>
       </c>
       <c r="E33" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F33" t="s">
         <v>140</v>

</xml_diff>